<commit_message>
Apply role-specific settlement access
</commit_message>
<xml_diff>
--- a/outputs/internal_accounts_20260715/Food-Fee_더미_사원_로그인_계정.xlsx
+++ b/outputs/internal_accounts_20260715/Food-Fee_더미_사원_로그인_계정.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="로그인 계정" sheetId="1" r:id="Rfbaea62f13684e8d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="로그인 계정" sheetId="1" r:id="R11ee90ef0e264855"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -281,7 +281,7 @@
         <x:color rgb="FF28785F"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -291,7 +291,7 @@
         <x:color rgb="FF64717D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF2F2F2"/>
         </x:patternFill>
       </x:fill>
@@ -302,7 +302,7 @@
         <x:color rgb="FF155866"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDDEBF7"/>
         </x:patternFill>
       </x:fill>
@@ -621,7 +621,7 @@
         <x:v>있음</x:v>
       </x:c>
       <x:c r="F6" s="37" t="str">
-        <x:v>있음</x:v>
+        <x:v>없음</x:v>
       </x:c>
       <x:c r="G6" s="37" t="str">
         <x:v>없음</x:v>
@@ -630,7 +630,7 @@
         <x:v>활성</x:v>
       </x:c>
       <x:c r="I6" s="39" t="str">
-        <x:v>정산 입력 및 Excel 출력 담당</x:v>
+        <x:v>현재 아이돌 식비 정산 전용 · 지급 정산금액/로그 비공개</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="28" customHeight="1">
@@ -641,26 +641,26 @@
         <x:v>상위 매니저</x:v>
       </x:c>
       <x:c r="C7" s="38" t="str">
-        <x:v>승인권자</x:v>
+        <x:v>상위 매니저</x:v>
       </x:c>
       <x:c r="D7" s="42" t="str">
         <x:f>RIGHT(A7,4)</x:f>
         <x:v>2201</x:v>
       </x:c>
       <x:c r="E7" s="38" t="str">
-        <x:v>없음</x:v>
+        <x:v>있음</x:v>
       </x:c>
       <x:c r="F7" s="38" t="str">
         <x:v>있음</x:v>
       </x:c>
       <x:c r="G7" s="38" t="str">
-        <x:v>있음</x:v>
+        <x:v>없음</x:v>
       </x:c>
       <x:c r="H7" s="38" t="str">
         <x:v>활성</x:v>
       </x:c>
       <x:c r="I7" s="40" t="str">
-        <x:v>승인 및 Excel 출력 담당</x:v>
+        <x:v>정산 입력·Excel 출력 가능 · 승인/로그 열람 불가</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="28" customHeight="1">
@@ -681,7 +681,7 @@
         <x:v>있음</x:v>
       </x:c>
       <x:c r="F8" s="38" t="str">
-        <x:v>없음</x:v>
+        <x:v>있음</x:v>
       </x:c>
       <x:c r="G8" s="38" t="str">
         <x:v>있음</x:v>
@@ -690,7 +690,7 @@
         <x:v>활성</x:v>
       </x:c>
       <x:c r="I8" s="40" t="str">
-        <x:v>인사 데이터 입력 및 승인 담당</x:v>
+        <x:v>모든 권한 보유 · 승인 버튼 및 감사 로그 열람 가능</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="26" customHeight="1">
@@ -769,7 +769,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rebff9e46e95a477f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5035155cbf79473b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>